<commit_message>
Corrige les erreurs #NOM? : remplace SOMME par SUM dans les formules
openpyxl exige les noms de fonctions en anglais (SUM, AVERAGE...).
Excel affiche automatiquement SOMME en français à l'ouverture.

https://claude.ai/code/session_01QQ9KiC56PBkHGrniFzX3y1
</commit_message>
<xml_diff>
--- a/TP_Indice_Gini_Deciles.xlsx
+++ b/TP_Indice_Gini_Deciles.xlsx
@@ -889,7 +889,7 @@
         <v/>
       </c>
       <c r="E5" s="8">
-        <f>SOMME($A$5:A5)/SOMME($A$5:$A$14)*100</f>
+        <f>SUM($A$5:A5)/SUM($A$5:$A$14)*100</f>
         <v/>
       </c>
       <c r="H5" s="9" t="inlineStr">
@@ -916,7 +916,7 @@
         <v/>
       </c>
       <c r="E6" s="8">
-        <f>SOMME($A$5:A6)/SOMME($A$5:$A$14)*100</f>
+        <f>SUM($A$5:A6)/SUM($A$5:$A$14)*100</f>
         <v/>
       </c>
       <c r="H6" s="10" t="inlineStr">
@@ -926,7 +926,7 @@
       </c>
       <c r="I6" s="11" t="n"/>
       <c r="J6" s="12">
-        <f>SOMME(A5:A14)</f>
+        <f>SUM(A5:A14)</f>
         <v/>
       </c>
       <c r="K6" s="11" t="n"/>
@@ -949,7 +949,7 @@
         <v/>
       </c>
       <c r="E7" s="8">
-        <f>SOMME($A$5:A7)/SOMME($A$5:$A$14)*100</f>
+        <f>SUM($A$5:A7)/SUM($A$5:$A$14)*100</f>
         <v/>
       </c>
       <c r="H7" s="10" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="I7" s="11" t="n"/>
       <c r="J7" s="12">
-        <f>SOMME(A5:A14)/10</f>
+        <f>SUM(A5:A14)/10</f>
         <v/>
       </c>
       <c r="K7" s="11" t="n"/>
@@ -982,7 +982,7 @@
         <v/>
       </c>
       <c r="E8" s="8">
-        <f>SOMME($A$5:A8)/SOMME($A$5:$A$14)*100</f>
+        <f>SUM($A$5:A8)/SUM($A$5:$A$14)*100</f>
         <v/>
       </c>
       <c r="H8" s="13" t="inlineStr">
@@ -1015,7 +1015,7 @@
         <v/>
       </c>
       <c r="E9" s="8">
-        <f>SOMME($A$5:A9)/SOMME($A$5:$A$14)*100</f>
+        <f>SUM($A$5:A9)/SUM($A$5:$A$14)*100</f>
         <v/>
       </c>
       <c r="H9" s="13" t="inlineStr">
@@ -1051,7 +1051,7 @@
         <v/>
       </c>
       <c r="E10" s="8">
-        <f>SOMME($A$5:A10)/SOMME($A$5:$A$14)*100</f>
+        <f>SUM($A$5:A10)/SUM($A$5:$A$14)*100</f>
         <v/>
       </c>
       <c r="H10" s="16" t="inlineStr">
@@ -1084,7 +1084,7 @@
         <v/>
       </c>
       <c r="E11" s="8">
-        <f>SOMME($A$5:A11)/SOMME($A$5:$A$14)*100</f>
+        <f>SUM($A$5:A11)/SUM($A$5:$A$14)*100</f>
         <v/>
       </c>
       <c r="M11" t="n">
@@ -1106,7 +1106,7 @@
         <v/>
       </c>
       <c r="E12" s="8">
-        <f>SOMME($A$5:A12)/SOMME($A$5:$A$14)*100</f>
+        <f>SUM($A$5:A12)/SUM($A$5:$A$14)*100</f>
         <v/>
       </c>
       <c r="H12" s="10" t="inlineStr">
@@ -1116,7 +1116,7 @@
       </c>
       <c r="I12" s="11" t="n"/>
       <c r="J12" s="18">
-        <f>0.05*(2*SOMME(E5:E13)/100+E14/100)</f>
+        <f>0.05*(2*SUM(E5:E13)/100+E14/100)</f>
         <v/>
       </c>
       <c r="K12" s="11" t="n"/>
@@ -1139,7 +1139,7 @@
         <v/>
       </c>
       <c r="E13" s="8">
-        <f>SOMME($A$5:A13)/SOMME($A$5:$A$14)*100</f>
+        <f>SUM($A$5:A13)/SUM($A$5:$A$14)*100</f>
         <v/>
       </c>
       <c r="H13" s="19" t="inlineStr">
@@ -1172,7 +1172,7 @@
         <v/>
       </c>
       <c r="E14" s="8">
-        <f>SOMME($A$5:A14)/SOMME($A$5:$A$14)*100</f>
+        <f>SUM($A$5:A14)/SUM($A$5:$A$14)*100</f>
         <v/>
       </c>
       <c r="H14" s="21" t="inlineStr">
@@ -1188,11 +1188,11 @@
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="22">
-        <f>SOMME(A5:A14)</f>
+        <f>SUM(A5:A14)</f>
         <v/>
       </c>
       <c r="C15" s="22">
-        <f>SOMME(C5:C14)</f>
+        <f>SUM(C5:C14)</f>
         <v/>
       </c>
       <c r="D15" s="22">

</xml_diff>

<commit_message>
Ajoute titre 'Courbe de Concentration' et signature Traore
- Graphique renommé en 'Courbe de Concentration'
- Signature 'Réalisé par : Traore' ajoutée en bas du tableau (ligne 20)

https://claude.ai/code/session_01QQ9KiC56PBkHGrniFzX3y1
</commit_message>
<xml_diff>
--- a/TP_Indice_Gini_Deciles.xlsx
+++ b/TP_Indice_Gini_Deciles.xlsx
@@ -22,7 +22,7 @@
     <numFmt numFmtId="166" formatCode="0 &quot;%&quot;"/>
     <numFmt numFmtId="167" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -83,6 +83,12 @@
       <i val="1"/>
       <color rgb="00000000"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="12">
@@ -189,7 +195,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -257,6 +263,9 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -347,7 +356,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Courbe de Lorenz</a:t>
+              <a:t>Courbe de Concentration</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -804,7 +813,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M18"/>
+  <dimension ref="A1:M20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1220,7 +1229,13 @@
       </c>
     </row>
     <row r="19" ht="18" customHeight="1"/>
-    <row r="20" ht="18" customHeight="1"/>
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" s="24" t="inlineStr">
+        <is>
+          <t>Réalisé par : Traore</t>
+        </is>
+      </c>
+    </row>
     <row r="21" ht="18" customHeight="1"/>
     <row r="22" ht="18" customHeight="1"/>
     <row r="23" ht="18" customHeight="1"/>
@@ -1241,7 +1256,7 @@
     <row r="38" ht="18" customHeight="1"/>
     <row r="39" ht="18" customHeight="1"/>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="21">
     <mergeCell ref="E1:M1"/>
     <mergeCell ref="H10:I10"/>
     <mergeCell ref="J10:K10"/>
@@ -1260,6 +1275,7 @@
     <mergeCell ref="H12:I12"/>
     <mergeCell ref="H14:K15"/>
     <mergeCell ref="J12:K12"/>
+    <mergeCell ref="A20:E20"/>
     <mergeCell ref="H8:I8"/>
     <mergeCell ref="J8:K8"/>
   </mergeCells>

</xml_diff>